<commit_message>
added tb after lib always
</commit_message>
<xml_diff>
--- a/tests/data/mock_b_and_t_cells_exp.xlsx
+++ b/tests/data/mock_b_and_t_cells_exp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabewilson/Desktop/worklist_generation/tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{471661DF-9C1C-0641-B062-566A46C4CC6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D90A10F-E59C-B54A-932A-41D8AEEC6ACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16860" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="106">
   <si>
     <t>Name:</t>
   </si>
@@ -312,6 +312,9 @@
     <t>tb</t>
   </si>
   <si>
+    <t>RA1</t>
+  </si>
+  <si>
     <t>Notes (not used):</t>
   </si>
   <si>
@@ -346,6 +349,9 @@
   </si>
   <si>
     <t>wetfile</t>
+  </si>
+  <si>
+    <t>No</t>
   </si>
 </sst>
 </file>
@@ -1289,7 +1295,7 @@
         <v>4</v>
       </c>
       <c r="AH1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="AM1" s="29"/>
       <c r="AO1" s="28"/>
@@ -1393,7 +1399,7 @@
         <v>30</v>
       </c>
       <c r="AJ4" s="6" t="s">
-        <v>31</v>
+        <v>105</v>
       </c>
       <c r="AK4" s="86" t="s">
         <v>32</v>
@@ -1498,11 +1504,13 @@
         <v>1</v>
       </c>
       <c r="AI5" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="AJ5" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="AK5" s="86" t="s">
         <v>96</v>
-      </c>
-      <c r="AJ5" s="6"/>
-      <c r="AK5" s="86" t="s">
-        <v>95</v>
       </c>
       <c r="AL5" s="91"/>
       <c r="AM5" s="9"/>
@@ -1789,7 +1797,7 @@
         <v>1</v>
       </c>
       <c r="AI8" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AJ8" s="19" t="s">
         <v>33</v>
@@ -1891,7 +1899,7 @@
         <v>1</v>
       </c>
       <c r="AI9" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AJ9" s="6"/>
       <c r="AK9" s="90"/>
@@ -6655,10 +6663,10 @@
       <c r="O12" s="10"/>
       <c r="P12" s="10"/>
       <c r="Q12" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
@@ -6706,7 +6714,7 @@
       <c r="O13" s="10"/>
       <c r="P13" s="10"/>
       <c r="Q13" s="82" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="R13" s="83"/>
     </row>
@@ -6741,10 +6749,10 @@
         <v>57</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K14" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L14" s="26">
         <f>IF(LEN(User!AG14)=0,"",User!AG14)</f>
@@ -6786,10 +6794,10 @@
         <v>57</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K15" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L15" s="26">
         <f>IF(LEN(User!AG15)=0,"",User!AG15)</f>
@@ -6831,10 +6839,10 @@
         <v>57</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="L16" s="26">
         <f>IF(LEN(User!AG16)=0,"",User!AG16)</f>

</xml_diff>

<commit_message>
Changed if statement for 1xp
</commit_message>
<xml_diff>
--- a/tests/data/mock_b_and_t_cells_exp.xlsx
+++ b/tests/data/mock_b_and_t_cells_exp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabewilson/Desktop/worklist_generation/tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D90A10F-E59C-B54A-932A-41D8AEEC6ACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08775FB9-5446-8B40-B544-03095727BCB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16860" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="16860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="105">
   <si>
     <t>Name:</t>
   </si>
@@ -349,9 +349,6 @@
   </si>
   <si>
     <t>wetfile</t>
-  </si>
-  <si>
-    <t>No</t>
   </si>
 </sst>
 </file>
@@ -1399,7 +1396,7 @@
         <v>30</v>
       </c>
       <c r="AJ4" s="6" t="s">
-        <v>105</v>
+        <v>31</v>
       </c>
       <c r="AK4" s="86" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
Walkthrough and README new
</commit_message>
<xml_diff>
--- a/tests/data/mock_b_and_t_cells_exp.xlsx
+++ b/tests/data/mock_b_and_t_cells_exp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabewilson/Desktop/worklist_generation/tests/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/01c1829094dbd390/Desktop/Kelly_Lab/.venv/worklist_git/tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B022A0-875C-C14E-8E37-79CB7BA39312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14680" yWindow="700" windowWidth="14720" windowHeight="16940" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User" sheetId="1" r:id="rId1"/>
@@ -857,6 +857,21 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -872,21 +887,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1237,7 +1237,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AU63"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="15.6640625" customWidth="1"/>
@@ -1260,7 +1260,7 @@
     <col min="43" max="45" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:47" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1285,7 +1285,7 @@
       <c r="AM1" s="29"/>
       <c r="AO1" s="28"/>
     </row>
-    <row r="2" spans="1:47" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:47" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -1312,7 +1312,7 @@
       <c r="AN2" s="9"/>
       <c r="AO2" s="28"/>
     </row>
-    <row r="3" spans="1:47" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:47" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -1340,7 +1340,7 @@
       <c r="AO3" s="28"/>
       <c r="AU3" s="21"/>
     </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:47" x14ac:dyDescent="0.4">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="D4" s="3"/>
@@ -1386,15 +1386,15 @@
       <c r="AJ4" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="AK4" s="81" t="s">
+      <c r="AK4" s="86" t="s">
         <v>32</v>
       </c>
-      <c r="AL4" s="82"/>
+      <c r="AL4" s="87"/>
       <c r="AM4" s="9"/>
       <c r="AN4" s="9"/>
       <c r="AO4" s="28"/>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:47" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
@@ -1494,15 +1494,15 @@
       <c r="AJ5" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="AK5" s="81" t="s">
+      <c r="AK5" s="86" t="s">
         <v>96</v>
       </c>
-      <c r="AL5" s="86"/>
+      <c r="AL5" s="91"/>
       <c r="AM5" s="9"/>
       <c r="AN5" s="9"/>
       <c r="AO5" s="28"/>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.4">
       <c r="A6" s="12" t="s">
         <v>12</v>
       </c>
@@ -1601,7 +1601,7 @@
       <c r="AN6" s="9"/>
       <c r="AO6" s="28"/>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:47" x14ac:dyDescent="0.4">
       <c r="D7" t="s">
         <v>14</v>
       </c>
@@ -1671,10 +1671,10 @@
       <c r="Z7" s="42">
         <v>4</v>
       </c>
-      <c r="AA7" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB7" s="89">
+      <c r="AA7" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB7" s="79">
         <v>14</v>
       </c>
       <c r="AD7" s="11">
@@ -1693,7 +1693,7 @@
       <c r="AN7" s="9"/>
       <c r="AO7" s="28"/>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.4">
       <c r="D8" t="s">
         <v>15</v>
       </c>
@@ -1763,10 +1763,10 @@
       <c r="Z8" s="42">
         <v>4</v>
       </c>
-      <c r="AA8" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB8" s="89">
+      <c r="AA8" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB8" s="79">
         <v>14</v>
       </c>
       <c r="AD8" s="11">
@@ -1787,15 +1787,15 @@
       <c r="AJ8" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="AK8" s="81" t="s">
+      <c r="AK8" s="86" t="s">
         <v>34</v>
       </c>
-      <c r="AL8" s="82"/>
+      <c r="AL8" s="87"/>
       <c r="AM8" s="9"/>
       <c r="AN8" s="9"/>
       <c r="AO8" s="28"/>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:47" x14ac:dyDescent="0.4">
       <c r="D9" t="s">
         <v>16</v>
       </c>
@@ -1865,10 +1865,10 @@
       <c r="Z9" s="42">
         <v>4</v>
       </c>
-      <c r="AA9" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB9" s="89">
+      <c r="AA9" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB9" s="79">
         <v>14</v>
       </c>
       <c r="AD9" s="11">
@@ -1887,13 +1887,13 @@
         <v>99</v>
       </c>
       <c r="AJ9" s="6"/>
-      <c r="AK9" s="85"/>
-      <c r="AL9" s="82"/>
+      <c r="AK9" s="90"/>
+      <c r="AL9" s="87"/>
       <c r="AM9" s="9"/>
       <c r="AN9" s="9"/>
       <c r="AO9" s="28"/>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:47" x14ac:dyDescent="0.4">
       <c r="D10" t="s">
         <v>17</v>
       </c>
@@ -1963,10 +1963,10 @@
       <c r="Z10" s="42">
         <v>4</v>
       </c>
-      <c r="AA10" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB10" s="89">
+      <c r="AA10" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB10" s="79">
         <v>14</v>
       </c>
       <c r="AD10" s="11">
@@ -1981,19 +1981,19 @@
       <c r="AG10" s="26">
         <v>1</v>
       </c>
-      <c r="AI10" s="83" t="s">
+      <c r="AI10" s="88" t="s">
         <v>35</v>
       </c>
-      <c r="AJ10" s="79" t="s">
+      <c r="AJ10" s="84" t="s">
         <v>31</v>
       </c>
-      <c r="AK10" s="85"/>
-      <c r="AL10" s="82"/>
+      <c r="AK10" s="90"/>
+      <c r="AL10" s="87"/>
       <c r="AM10" s="9"/>
       <c r="AN10" s="9"/>
       <c r="AO10" s="28"/>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:47" x14ac:dyDescent="0.4">
       <c r="D11" t="s">
         <v>18</v>
       </c>
@@ -2063,10 +2063,10 @@
       <c r="Z11" s="42">
         <v>4</v>
       </c>
-      <c r="AA11" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB11" s="89">
+      <c r="AA11" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB11" s="79">
         <v>14</v>
       </c>
       <c r="AD11" s="11">
@@ -2081,15 +2081,15 @@
       <c r="AG11" s="26">
         <v>1</v>
       </c>
-      <c r="AI11" s="84"/>
-      <c r="AJ11" s="80"/>
+      <c r="AI11" s="89"/>
+      <c r="AJ11" s="85"/>
       <c r="AK11" s="30"/>
       <c r="AL11" s="30"/>
       <c r="AM11" s="9"/>
       <c r="AN11" s="9"/>
       <c r="AO11" s="28"/>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:47" x14ac:dyDescent="0.4">
       <c r="D12" t="s">
         <v>19</v>
       </c>
@@ -2159,10 +2159,10 @@
       <c r="Z12" s="42">
         <v>4</v>
       </c>
-      <c r="AA12" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB12" s="89">
+      <c r="AA12" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB12" s="79">
         <v>14</v>
       </c>
       <c r="AD12" s="11">
@@ -2185,7 +2185,7 @@
       <c r="AN12" s="9"/>
       <c r="AO12" s="28"/>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.4">
       <c r="D13" t="s">
         <v>20</v>
       </c>
@@ -2255,10 +2255,10 @@
       <c r="Z13" s="42">
         <v>4</v>
       </c>
-      <c r="AA13" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB13" s="89">
+      <c r="AA13" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB13" s="79">
         <v>14</v>
       </c>
       <c r="AD13" s="11">
@@ -2281,7 +2281,7 @@
       <c r="AN13" s="9"/>
       <c r="AO13" s="28"/>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.4">
       <c r="D14" t="s">
         <v>21</v>
       </c>
@@ -2351,10 +2351,10 @@
       <c r="Z14" s="42">
         <v>4</v>
       </c>
-      <c r="AA14" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB14" s="89">
+      <c r="AA14" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB14" s="79">
         <v>14</v>
       </c>
       <c r="AD14" s="11">
@@ -2377,7 +2377,7 @@
       <c r="AN14" s="9"/>
       <c r="AO14" s="28"/>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.4">
       <c r="D15" t="s">
         <v>22</v>
       </c>
@@ -2447,10 +2447,10 @@
       <c r="Z15" s="42">
         <v>4</v>
       </c>
-      <c r="AA15" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB15" s="89">
+      <c r="AA15" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB15" s="79">
         <v>14</v>
       </c>
       <c r="AD15" s="11">
@@ -2459,7 +2459,7 @@
       <c r="AE15" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="AF15" s="91" t="s">
+      <c r="AF15" s="81" t="s">
         <v>72</v>
       </c>
       <c r="AG15" s="26">
@@ -2473,7 +2473,7 @@
       <c r="AN15" s="9"/>
       <c r="AO15" s="28"/>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:47" x14ac:dyDescent="0.4">
       <c r="D16" t="s">
         <v>23</v>
       </c>
@@ -2543,10 +2543,10 @@
       <c r="Z16" s="42">
         <v>4</v>
       </c>
-      <c r="AA16" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB16" s="89">
+      <c r="AA16" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB16" s="79">
         <v>14</v>
       </c>
       <c r="AD16" s="11">
@@ -2569,7 +2569,7 @@
       <c r="AN16" s="9"/>
       <c r="AO16" s="28"/>
     </row>
-    <row r="17" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D17" t="s">
         <v>24</v>
       </c>
@@ -2639,10 +2639,10 @@
       <c r="Z17" s="42">
         <v>4</v>
       </c>
-      <c r="AA17" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB17" s="89">
+      <c r="AA17" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB17" s="79">
         <v>14</v>
       </c>
       <c r="AD17" s="11">
@@ -2664,7 +2664,7 @@
       <c r="AN17" s="9"/>
       <c r="AO17" s="28"/>
     </row>
-    <row r="18" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D18" t="s">
         <v>25</v>
       </c>
@@ -2734,10 +2734,10 @@
       <c r="Z18" s="42">
         <v>4</v>
       </c>
-      <c r="AA18" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB18" s="89">
+      <c r="AA18" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB18" s="79">
         <v>14</v>
       </c>
       <c r="AD18" s="11">
@@ -2753,7 +2753,7 @@
       <c r="AN18" s="9"/>
       <c r="AO18" s="28"/>
     </row>
-    <row r="19" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D19" t="s">
         <v>26</v>
       </c>
@@ -2823,10 +2823,10 @@
       <c r="Z19" s="42">
         <v>4</v>
       </c>
-      <c r="AA19" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB19" s="89">
+      <c r="AA19" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB19" s="79">
         <v>14</v>
       </c>
       <c r="AD19" s="11">
@@ -2839,7 +2839,7 @@
       <c r="AN19" s="9"/>
       <c r="AO19" s="28"/>
     </row>
-    <row r="20" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D20" t="s">
         <v>27</v>
       </c>
@@ -2909,10 +2909,10 @@
       <c r="Z20" s="42">
         <v>4</v>
       </c>
-      <c r="AA20" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB20" s="89">
+      <c r="AA20" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB20" s="79">
         <v>14</v>
       </c>
       <c r="AD20" s="11">
@@ -2925,7 +2925,7 @@
       <c r="AN20" s="9"/>
       <c r="AO20" s="28"/>
     </row>
-    <row r="21" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D21" t="s">
         <v>28</v>
       </c>
@@ -3011,7 +3011,7 @@
       <c r="AN21" s="9"/>
       <c r="AO21" s="28"/>
     </row>
-    <row r="22" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="D22" s="3"/>
@@ -3049,7 +3049,7 @@
       <c r="AN22" s="9"/>
       <c r="AO22" s="28"/>
     </row>
-    <row r="23" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A23" s="4" t="s">
         <v>9</v>
       </c>
@@ -3145,7 +3145,7 @@
       <c r="AN23" s="9"/>
       <c r="AO23" s="28"/>
     </row>
-    <row r="24" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A24" s="12" t="s">
         <v>19</v>
       </c>
@@ -3241,7 +3241,7 @@
       <c r="AN24" s="9"/>
       <c r="AO24" s="28"/>
     </row>
-    <row r="25" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D25" t="s">
         <v>14</v>
       </c>
@@ -3311,10 +3311,10 @@
       <c r="Z25" s="62">
         <v>8</v>
       </c>
-      <c r="AA25" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB25" s="90">
+      <c r="AA25" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB25" s="80">
         <v>14</v>
       </c>
       <c r="AD25" s="11">
@@ -3331,7 +3331,7 @@
       <c r="AN25" s="9"/>
       <c r="AO25" s="28"/>
     </row>
-    <row r="26" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D26" t="s">
         <v>15</v>
       </c>
@@ -3401,10 +3401,10 @@
       <c r="Z26" s="62">
         <v>8</v>
       </c>
-      <c r="AA26" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB26" s="90">
+      <c r="AA26" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB26" s="80">
         <v>14</v>
       </c>
       <c r="AD26" s="11">
@@ -3421,7 +3421,7 @@
       <c r="AN26" s="9"/>
       <c r="AO26" s="28"/>
     </row>
-    <row r="27" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D27" t="s">
         <v>16</v>
       </c>
@@ -3491,10 +3491,10 @@
       <c r="Z27" s="62">
         <v>8</v>
       </c>
-      <c r="AA27" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB27" s="90">
+      <c r="AA27" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB27" s="80">
         <v>14</v>
       </c>
       <c r="AD27" s="11">
@@ -3511,7 +3511,7 @@
       <c r="AN27" s="9"/>
       <c r="AO27" s="28"/>
     </row>
-    <row r="28" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D28" t="s">
         <v>17</v>
       </c>
@@ -3581,10 +3581,10 @@
       <c r="Z28" s="62">
         <v>8</v>
       </c>
-      <c r="AA28" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB28" s="90">
+      <c r="AA28" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB28" s="80">
         <v>14</v>
       </c>
       <c r="AD28" s="11">
@@ -3601,7 +3601,7 @@
       <c r="AN28" s="9"/>
       <c r="AO28" s="28"/>
     </row>
-    <row r="29" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D29" t="s">
         <v>18</v>
       </c>
@@ -3671,10 +3671,10 @@
       <c r="Z29" s="62">
         <v>8</v>
       </c>
-      <c r="AA29" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB29" s="90">
+      <c r="AA29" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB29" s="80">
         <v>14</v>
       </c>
       <c r="AD29" s="11">
@@ -3691,7 +3691,7 @@
       <c r="AN29" s="9"/>
       <c r="AO29" s="28"/>
     </row>
-    <row r="30" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D30" t="s">
         <v>19</v>
       </c>
@@ -3761,10 +3761,10 @@
       <c r="Z30" s="62">
         <v>8</v>
       </c>
-      <c r="AA30" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB30" s="90">
+      <c r="AA30" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB30" s="80">
         <v>14</v>
       </c>
       <c r="AD30" s="11">
@@ -3781,7 +3781,7 @@
       <c r="AN30" s="9"/>
       <c r="AO30" s="28"/>
     </row>
-    <row r="31" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D31" t="s">
         <v>20</v>
       </c>
@@ -3851,10 +3851,10 @@
       <c r="Z31" s="62">
         <v>8</v>
       </c>
-      <c r="AA31" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB31" s="90">
+      <c r="AA31" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB31" s="80">
         <v>14</v>
       </c>
       <c r="AD31" s="11">
@@ -3871,7 +3871,7 @@
       <c r="AN31" s="9"/>
       <c r="AO31" s="28"/>
     </row>
-    <row r="32" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D32" t="s">
         <v>21</v>
       </c>
@@ -3941,10 +3941,10 @@
       <c r="Z32" s="62">
         <v>8</v>
       </c>
-      <c r="AA32" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB32" s="90">
+      <c r="AA32" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB32" s="80">
         <v>14</v>
       </c>
       <c r="AD32" s="11">
@@ -3961,7 +3961,7 @@
       <c r="AN32" s="9"/>
       <c r="AO32" s="28"/>
     </row>
-    <row r="33" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D33" t="s">
         <v>22</v>
       </c>
@@ -4031,10 +4031,10 @@
       <c r="Z33" s="62">
         <v>8</v>
       </c>
-      <c r="AA33" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB33" s="90">
+      <c r="AA33" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB33" s="80">
         <v>14</v>
       </c>
       <c r="AD33" s="11">
@@ -4047,7 +4047,7 @@
       <c r="AN33" s="9"/>
       <c r="AO33" s="28"/>
     </row>
-    <row r="34" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D34" t="s">
         <v>23</v>
       </c>
@@ -4117,10 +4117,10 @@
       <c r="Z34" s="62">
         <v>8</v>
       </c>
-      <c r="AA34" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB34" s="90">
+      <c r="AA34" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB34" s="80">
         <v>14</v>
       </c>
       <c r="AD34" s="11">
@@ -4130,7 +4130,7 @@
       <c r="AF34" s="10"/>
       <c r="AG34" s="10"/>
     </row>
-    <row r="35" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D35" t="s">
         <v>24</v>
       </c>
@@ -4200,10 +4200,10 @@
       <c r="Z35" s="62">
         <v>8</v>
       </c>
-      <c r="AA35" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB35" s="90">
+      <c r="AA35" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB35" s="80">
         <v>14</v>
       </c>
       <c r="AD35" s="11">
@@ -4213,7 +4213,7 @@
       <c r="AF35" s="10"/>
       <c r="AG35" s="10"/>
     </row>
-    <row r="36" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D36" t="s">
         <v>25</v>
       </c>
@@ -4283,10 +4283,10 @@
       <c r="Z36" s="62">
         <v>8</v>
       </c>
-      <c r="AA36" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB36" s="90">
+      <c r="AA36" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB36" s="80">
         <v>14</v>
       </c>
       <c r="AD36" s="11">
@@ -4296,7 +4296,7 @@
       <c r="AF36" s="10"/>
       <c r="AG36" s="10"/>
     </row>
-    <row r="37" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D37" t="s">
         <v>26</v>
       </c>
@@ -4366,10 +4366,10 @@
       <c r="Z37" s="62">
         <v>8</v>
       </c>
-      <c r="AA37" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB37" s="90">
+      <c r="AA37" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB37" s="80">
         <v>14</v>
       </c>
       <c r="AD37" s="11">
@@ -4379,7 +4379,7 @@
       <c r="AF37" s="10"/>
       <c r="AG37" s="10"/>
     </row>
-    <row r="38" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D38" t="s">
         <v>27</v>
       </c>
@@ -4449,10 +4449,10 @@
       <c r="Z38" s="62">
         <v>8</v>
       </c>
-      <c r="AA38" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB38" s="90">
+      <c r="AA38" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB38" s="80">
         <v>14</v>
       </c>
       <c r="AD38" s="11">
@@ -4462,7 +4462,7 @@
       <c r="AF38" s="10"/>
       <c r="AG38" s="10"/>
     </row>
-    <row r="39" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D39" t="s">
         <v>28</v>
       </c>
@@ -4545,7 +4545,7 @@
       <c r="AF39" s="10"/>
       <c r="AG39" s="10"/>
     </row>
-    <row r="40" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="D40" s="3"/>
@@ -4582,7 +4582,7 @@
       <c r="AJ40" s="30"/>
       <c r="AK40" s="30"/>
     </row>
-    <row r="41" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A41" s="4" t="s">
         <v>9</v>
       </c>
@@ -4673,7 +4673,7 @@
       <c r="AJ41" s="30"/>
       <c r="AK41" s="30"/>
     </row>
-    <row r="42" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:41" x14ac:dyDescent="0.4">
       <c r="A42" s="12" t="s">
         <v>14</v>
       </c>
@@ -4762,7 +4762,7 @@
       <c r="AF42" s="10"/>
       <c r="AG42" s="10"/>
     </row>
-    <row r="43" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D43" t="s">
         <v>14</v>
       </c>
@@ -4832,10 +4832,10 @@
       <c r="Z43" s="50">
         <v>12</v>
       </c>
-      <c r="AA43" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB43" s="89">
+      <c r="AA43" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB43" s="79">
         <v>14</v>
       </c>
       <c r="AD43" s="11">
@@ -4845,7 +4845,7 @@
       <c r="AF43" s="10"/>
       <c r="AG43" s="10"/>
     </row>
-    <row r="44" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D44" t="s">
         <v>15</v>
       </c>
@@ -4915,10 +4915,10 @@
       <c r="Z44" s="50">
         <v>12</v>
       </c>
-      <c r="AA44" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB44" s="89">
+      <c r="AA44" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB44" s="79">
         <v>14</v>
       </c>
       <c r="AD44" s="11">
@@ -4928,7 +4928,7 @@
       <c r="AF44" s="10"/>
       <c r="AG44" s="10"/>
     </row>
-    <row r="45" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:41" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D45" t="s">
         <v>16</v>
       </c>
@@ -4998,10 +4998,10 @@
       <c r="Z45" s="50">
         <v>12</v>
       </c>
-      <c r="AA45" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB45" s="89">
+      <c r="AA45" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB45" s="79">
         <v>14</v>
       </c>
       <c r="AD45" s="11">
@@ -5011,7 +5011,7 @@
       <c r="AF45" s="10"/>
       <c r="AG45" s="10"/>
     </row>
-    <row r="46" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D46" t="s">
         <v>17</v>
       </c>
@@ -5081,10 +5081,10 @@
       <c r="Z46" s="50">
         <v>12</v>
       </c>
-      <c r="AA46" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB46" s="89">
+      <c r="AA46" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB46" s="79">
         <v>14</v>
       </c>
       <c r="AD46" s="11">
@@ -5094,7 +5094,7 @@
       <c r="AF46" s="10"/>
       <c r="AG46" s="10"/>
     </row>
-    <row r="47" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D47" t="s">
         <v>18</v>
       </c>
@@ -5164,10 +5164,10 @@
       <c r="Z47" s="50">
         <v>12</v>
       </c>
-      <c r="AA47" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB47" s="89">
+      <c r="AA47" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB47" s="79">
         <v>14</v>
       </c>
       <c r="AD47" s="11">
@@ -5177,7 +5177,7 @@
       <c r="AF47" s="10"/>
       <c r="AG47" s="10"/>
     </row>
-    <row r="48" spans="1:41" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:41" x14ac:dyDescent="0.4">
       <c r="D48" t="s">
         <v>19</v>
       </c>
@@ -5247,10 +5247,10 @@
       <c r="Z48" s="50">
         <v>12</v>
       </c>
-      <c r="AA48" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB48" s="89">
+      <c r="AA48" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB48" s="79">
         <v>14</v>
       </c>
       <c r="AD48" s="11">
@@ -5260,7 +5260,7 @@
       <c r="AF48" s="24"/>
       <c r="AG48" s="10"/>
     </row>
-    <row r="49" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:40" x14ac:dyDescent="0.4">
       <c r="D49" t="s">
         <v>20</v>
       </c>
@@ -5330,10 +5330,10 @@
       <c r="Z49" s="50">
         <v>12</v>
       </c>
-      <c r="AA49" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB49" s="89">
+      <c r="AA49" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB49" s="79">
         <v>14</v>
       </c>
       <c r="AD49" s="11">
@@ -5343,7 +5343,7 @@
       <c r="AF49" s="24"/>
       <c r="AG49" s="10"/>
     </row>
-    <row r="50" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:40" x14ac:dyDescent="0.4">
       <c r="D50" t="s">
         <v>21</v>
       </c>
@@ -5413,10 +5413,10 @@
       <c r="Z50" s="50">
         <v>12</v>
       </c>
-      <c r="AA50" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB50" s="89">
+      <c r="AA50" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB50" s="79">
         <v>14</v>
       </c>
       <c r="AD50" s="11">
@@ -5426,7 +5426,7 @@
       <c r="AF50" s="24"/>
       <c r="AG50" s="10"/>
     </row>
-    <row r="51" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:40" x14ac:dyDescent="0.4">
       <c r="D51" t="s">
         <v>22</v>
       </c>
@@ -5496,10 +5496,10 @@
       <c r="Z51" s="50">
         <v>12</v>
       </c>
-      <c r="AA51" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB51" s="89">
+      <c r="AA51" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB51" s="79">
         <v>14</v>
       </c>
       <c r="AD51" s="17">
@@ -5509,7 +5509,7 @@
       <c r="AF51" s="18"/>
       <c r="AG51" s="18"/>
     </row>
-    <row r="52" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:40" x14ac:dyDescent="0.4">
       <c r="D52" t="s">
         <v>23</v>
       </c>
@@ -5579,14 +5579,14 @@
       <c r="Z52" s="50">
         <v>12</v>
       </c>
-      <c r="AA52" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB52" s="89">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="53" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AA52" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB52" s="79">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="53" spans="1:40" x14ac:dyDescent="0.4">
       <c r="D53" t="s">
         <v>24</v>
       </c>
@@ -5656,10 +5656,10 @@
       <c r="Z53" s="50">
         <v>12</v>
       </c>
-      <c r="AA53" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB53" s="89">
+      <c r="AA53" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB53" s="79">
         <v>14</v>
       </c>
       <c r="AE53" s="20"/>
@@ -5667,7 +5667,7 @@
       <c r="AM53" s="20"/>
       <c r="AN53" s="20"/>
     </row>
-    <row r="54" spans="1:40" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:40" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D54" t="s">
         <v>25</v>
       </c>
@@ -5737,10 +5737,10 @@
       <c r="Z54" s="50">
         <v>12</v>
       </c>
-      <c r="AA54" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB54" s="89">
+      <c r="AA54" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB54" s="79">
         <v>14</v>
       </c>
       <c r="AE54" s="20"/>
@@ -5748,7 +5748,7 @@
       <c r="AM54" s="20"/>
       <c r="AN54" s="20"/>
     </row>
-    <row r="55" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:40" x14ac:dyDescent="0.4">
       <c r="D55" t="s">
         <v>26</v>
       </c>
@@ -5818,10 +5818,10 @@
       <c r="Z55" s="50">
         <v>12</v>
       </c>
-      <c r="AA55" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB55" s="89">
+      <c r="AA55" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB55" s="79">
         <v>14</v>
       </c>
       <c r="AE55" s="20"/>
@@ -5829,7 +5829,7 @@
       <c r="AM55" s="20"/>
       <c r="AN55" s="20"/>
     </row>
-    <row r="56" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:40" x14ac:dyDescent="0.4">
       <c r="D56" t="s">
         <v>27</v>
       </c>
@@ -5899,15 +5899,15 @@
       <c r="Z56" s="50">
         <v>12</v>
       </c>
-      <c r="AA56" s="89">
-        <v>14</v>
-      </c>
-      <c r="AB56" s="89">
+      <c r="AA56" s="79">
+        <v>14</v>
+      </c>
+      <c r="AB56" s="79">
         <v>14</v>
       </c>
       <c r="AE56" s="9"/>
     </row>
-    <row r="57" spans="1:40" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:40" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="D57" t="s">
         <v>28</v>
       </c>
@@ -5989,7 +5989,7 @@
       <c r="AM57" s="20"/>
       <c r="AN57" s="20"/>
     </row>
-    <row r="58" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="D58" s="3"/>
@@ -6023,23 +6023,23 @@
       <c r="AM58" s="20"/>
       <c r="AN58" s="20"/>
     </row>
-    <row r="59" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:40" x14ac:dyDescent="0.4">
       <c r="AE59" s="9"/>
       <c r="AK59" s="20"/>
       <c r="AL59" s="21"/>
       <c r="AM59" s="20"/>
       <c r="AN59" s="20"/>
     </row>
-    <row r="60" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:40" x14ac:dyDescent="0.4">
       <c r="AE60" s="9"/>
     </row>
-    <row r="61" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:40" x14ac:dyDescent="0.4">
       <c r="AE61" s="9"/>
     </row>
-    <row r="62" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:40" x14ac:dyDescent="0.4">
       <c r="AE62" s="9"/>
     </row>
-    <row r="63" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:40" x14ac:dyDescent="0.4">
       <c r="AE63" s="9"/>
     </row>
   </sheetData>
@@ -6069,7 +6069,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="14" max="16" width="10.6640625" customWidth="1"/>
     <col min="17" max="17" width="30.83203125" customWidth="1"/>
@@ -6077,7 +6077,7 @@
     <col min="19" max="19" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A1" s="5" t="s">
         <v>1</v>
       </c>
@@ -6127,7 +6127,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A2" s="11">
         <v>1</v>
       </c>
@@ -6178,7 +6178,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A3" s="11">
         <v>2</v>
       </c>
@@ -6223,7 +6223,7 @@
       <c r="O3" s="10"/>
       <c r="P3" s="10"/>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A4" s="11">
         <v>3</v>
       </c>
@@ -6270,7 +6270,7 @@
       <c r="Q4" s="20"/>
       <c r="R4" s="21"/>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A5" s="11">
         <v>4</v>
       </c>
@@ -6321,7 +6321,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A6" s="11">
         <v>5</v>
       </c>
@@ -6366,7 +6366,7 @@
       <c r="O6" s="10"/>
       <c r="P6" s="10"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A7" s="11">
         <v>6</v>
       </c>
@@ -6411,7 +6411,7 @@
       <c r="O7" s="10"/>
       <c r="P7" s="10"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A8" s="11">
         <v>7</v>
       </c>
@@ -6462,7 +6462,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A9" s="11">
         <v>8</v>
       </c>
@@ -6513,7 +6513,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A10" s="11">
         <v>9</v>
       </c>
@@ -6558,7 +6558,7 @@
       <c r="O10" s="10"/>
       <c r="P10" s="10"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A11" s="11">
         <v>10</v>
       </c>
@@ -6603,7 +6603,7 @@
       <c r="O11" s="10"/>
       <c r="P11" s="10"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A12" s="11">
         <v>11</v>
       </c>
@@ -6654,7 +6654,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A13" s="11">
         <v>12</v>
       </c>
@@ -6698,12 +6698,12 @@
       <c r="N13" s="11"/>
       <c r="O13" s="10"/>
       <c r="P13" s="10"/>
-      <c r="Q13" s="87" t="s">
+      <c r="Q13" s="82" t="s">
         <v>94</v>
       </c>
-      <c r="R13" s="88"/>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="R13" s="83"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A14" s="11">
         <v>13</v>
       </c>
@@ -6748,7 +6748,7 @@
       <c r="O14" s="10"/>
       <c r="P14" s="10"/>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.4">
       <c r="A15" s="11">
         <v>14</v>
       </c>
@@ -6793,7 +6793,7 @@
       <c r="O15" s="10"/>
       <c r="P15" s="10"/>
     </row>
-    <row r="16" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="11">
         <v>15</v>
       </c>
@@ -6838,7 +6838,7 @@
       <c r="O16" s="10"/>
       <c r="P16" s="10"/>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A17" s="11">
         <v>16</v>
       </c>
@@ -6883,7 +6883,7 @@
       <c r="O17" s="10"/>
       <c r="P17" s="10"/>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A18" s="11">
         <v>17</v>
       </c>
@@ -6909,7 +6909,7 @@
       <c r="O18" s="10"/>
       <c r="P18" s="10"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A19" s="11">
         <v>18</v>
       </c>
@@ -6938,7 +6938,7 @@
       <c r="O19" s="10"/>
       <c r="P19" s="10"/>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A20" s="11">
         <v>19</v>
       </c>
@@ -6967,7 +6967,7 @@
       <c r="O20" s="10"/>
       <c r="P20" s="10"/>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A21" s="11">
         <v>20</v>
       </c>
@@ -6996,7 +6996,7 @@
       <c r="O21" s="10"/>
       <c r="P21" s="10"/>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A22" s="11">
         <v>21</v>
       </c>
@@ -7025,7 +7025,7 @@
       <c r="O22" s="10"/>
       <c r="P22" s="10"/>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A23" s="11">
         <v>22</v>
       </c>
@@ -7054,7 +7054,7 @@
       <c r="O23" s="10"/>
       <c r="P23" s="10"/>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A24" s="11">
         <v>23</v>
       </c>
@@ -7083,7 +7083,7 @@
       <c r="O24" s="10"/>
       <c r="P24" s="10"/>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A25" s="11">
         <v>24</v>
       </c>
@@ -7112,7 +7112,7 @@
       <c r="O25" s="10"/>
       <c r="P25" s="10"/>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A26" s="11">
         <v>25</v>
       </c>
@@ -7141,7 +7141,7 @@
       <c r="O26" s="10"/>
       <c r="P26" s="10"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A27" s="11">
         <v>26</v>
       </c>
@@ -7170,7 +7170,7 @@
       <c r="O27" s="10"/>
       <c r="P27" s="10"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A28" s="11">
         <v>27</v>
       </c>
@@ -7199,7 +7199,7 @@
       <c r="O28" s="10"/>
       <c r="P28" s="10"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A29" s="11">
         <v>28</v>
       </c>
@@ -7228,7 +7228,7 @@
       <c r="O29" s="10"/>
       <c r="P29" s="10"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A30" s="11">
         <v>29</v>
       </c>
@@ -7257,7 +7257,7 @@
       <c r="O30" s="10"/>
       <c r="P30" s="10"/>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A31" s="11">
         <v>30</v>
       </c>
@@ -7286,7 +7286,7 @@
       <c r="O31" s="10"/>
       <c r="P31" s="10"/>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A32" s="11">
         <v>31</v>
       </c>
@@ -7315,7 +7315,7 @@
       <c r="O32" s="10"/>
       <c r="P32" s="10"/>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A33" s="11">
         <v>32</v>
       </c>
@@ -7344,7 +7344,7 @@
       <c r="O33" s="10"/>
       <c r="P33" s="10"/>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A34" s="11">
         <v>33</v>
       </c>
@@ -7373,7 +7373,7 @@
       <c r="O34" s="10"/>
       <c r="P34" s="10"/>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A35" s="11">
         <v>34</v>
       </c>
@@ -7402,7 +7402,7 @@
       <c r="O35" s="10"/>
       <c r="P35" s="10"/>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A36" s="11">
         <v>35</v>
       </c>
@@ -7430,7 +7430,7 @@
       <c r="O36" s="10"/>
       <c r="P36" s="10"/>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A37" s="11">
         <v>36</v>
       </c>
@@ -7459,7 +7459,7 @@
       <c r="O37" s="10"/>
       <c r="P37" s="10"/>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A38" s="11">
         <v>37</v>
       </c>
@@ -7488,7 +7488,7 @@
       <c r="O38" s="10"/>
       <c r="P38" s="10"/>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A39" s="11">
         <v>38</v>
       </c>
@@ -7517,7 +7517,7 @@
       <c r="O39" s="10"/>
       <c r="P39" s="10"/>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A40" s="11">
         <v>39</v>
       </c>
@@ -7546,7 +7546,7 @@
       <c r="O40" s="10"/>
       <c r="P40" s="10"/>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A41" s="11">
         <v>40</v>
       </c>
@@ -7575,7 +7575,7 @@
       <c r="O41" s="10"/>
       <c r="P41" s="10"/>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A42" s="11">
         <v>41</v>
       </c>
@@ -7604,7 +7604,7 @@
       <c r="O42" s="10"/>
       <c r="P42" s="10"/>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A43" s="11">
         <v>42</v>
       </c>
@@ -7633,7 +7633,7 @@
       <c r="O43" s="10"/>
       <c r="P43" s="10"/>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A44" s="11">
         <v>43</v>
       </c>
@@ -7662,7 +7662,7 @@
       <c r="O44" s="10"/>
       <c r="P44" s="10"/>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A45" s="11">
         <v>44</v>
       </c>
@@ -7691,7 +7691,7 @@
       <c r="O45" s="10"/>
       <c r="P45" s="10"/>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A46" s="11">
         <v>45</v>
       </c>
@@ -7720,7 +7720,7 @@
       <c r="O46" s="10"/>
       <c r="P46" s="10"/>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A47" s="11">
         <v>46</v>
       </c>
@@ -7749,7 +7749,7 @@
       <c r="O47" s="10"/>
       <c r="P47" s="10"/>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A48" s="11">
         <v>47</v>
       </c>
@@ -7778,7 +7778,7 @@
       <c r="O48" s="10"/>
       <c r="P48" s="10"/>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A49" s="11">
         <v>48</v>
       </c>
@@ -7807,7 +7807,7 @@
       <c r="O49" s="10"/>
       <c r="P49" s="10"/>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A50" s="11">
         <v>49</v>
       </c>
@@ -7836,7 +7836,7 @@
       <c r="O50" s="10"/>
       <c r="P50" s="10"/>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.4">
       <c r="A51" s="17">
         <v>50</v>
       </c>

</xml_diff>